<commit_message>
extract psmart to legacy
</commit_message>
<xml_diff>
--- a/modules.xlsx
+++ b/modules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\josh\kenyaEMR-modules-updater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BD5A41-01D6-49C3-B383-4D840EBA127D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434E4C1F-63B6-4BC4-AB7D-22751BB99743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7576F9BB-DBC4-4D03-8B1C-D88545B56239}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$31</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="71">
   <si>
     <t>modules</t>
   </si>
@@ -103,9 +103,6 @@
     <t>kenyaemrorderentry</t>
   </si>
   <si>
-    <t>kenyaemrpsmart</t>
-  </si>
-  <si>
     <t>kenyakeypop</t>
   </si>
   <si>
@@ -215,9 +212,6 @@
   </si>
   <si>
     <t>https://github.com/palladiumkenya/openmrs-module-kenyaemrorderentry.git</t>
-  </si>
-  <si>
-    <t>https://github.com/palladiumkenya/openmrs-module-kenyaemrpsmart.git</t>
   </si>
   <si>
     <t>https://github.com/palladiumkenya/openmrs-module-kenyakeypop.git</t>
@@ -619,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D447332-634A-4264-831A-AFF551D7ED1B}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" bestFit="1" customWidth="1"/>
@@ -632,13 +626,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" t="s">
-        <v>33</v>
-      </c>
       <c r="D1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -646,10 +640,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -657,10 +651,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
         <v>36</v>
-      </c>
-      <c r="C3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -668,10 +662,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -679,10 +673,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -690,10 +684,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
         <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -701,10 +695,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -712,10 +706,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -723,10 +717,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -734,10 +728,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" t="s">
         <v>45</v>
-      </c>
-      <c r="C10" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -745,10 +739,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -756,10 +750,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
         <v>48</v>
-      </c>
-      <c r="C12" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -767,10 +761,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -778,10 +772,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -789,10 +783,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -800,10 +794,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -811,10 +805,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -822,10 +816,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -833,10 +827,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -844,10 +838,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -855,10 +849,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -866,10 +860,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -877,10 +871,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -888,10 +882,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C24" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -899,10 +893,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -910,10 +904,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C26" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -921,10 +915,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -932,10 +926,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" t="s">
         <v>65</v>
-      </c>
-      <c r="C28" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -943,10 +937,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -954,10 +948,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -968,22 +962,11 @@
         <v>68</v>
       </c>
       <c r="C31" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D32" xr:uid="{9D447332-634A-4264-831A-AFF551D7ED1B}"/>
+  <autoFilter ref="A1:D31" xr:uid="{9D447332-634A-4264-831A-AFF551D7ED1B}"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{FB795B93-36B6-46BF-94E9-0038AB747753}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{9B7024D0-965C-4E36-8BBD-D2B5693F8066}"/>
@@ -1005,17 +988,16 @@
     <hyperlink ref="B19" r:id="rId18" xr:uid="{CEFE724D-0289-4516-B679-5972075F9D45}"/>
     <hyperlink ref="B20" r:id="rId19" xr:uid="{9E0376B5-01C2-4493-9DBE-E1898317C082}"/>
     <hyperlink ref="B21" r:id="rId20" xr:uid="{5114C9EC-EEB3-4299-A9FD-2983F25CB21B}"/>
-    <hyperlink ref="B22" r:id="rId21" xr:uid="{8C48509F-21F4-4173-8B17-421ACD5D169D}"/>
-    <hyperlink ref="B23" r:id="rId22" xr:uid="{A430A9C6-FD58-4DE8-82B1-C2BDC43CD75D}"/>
-    <hyperlink ref="B24" r:id="rId23" xr:uid="{4BA87FC2-2482-47F3-AF0B-26573751D1D0}"/>
-    <hyperlink ref="B25" r:id="rId24" xr:uid="{CF736F36-5C13-46BF-8EFE-00A8F71CDBFA}"/>
-    <hyperlink ref="B26" r:id="rId25" xr:uid="{F3EE1F0F-3E4B-4FFA-A948-D718624032D3}"/>
-    <hyperlink ref="B27" r:id="rId26" xr:uid="{24CA94E5-1C41-4A90-8A88-F60639278F60}"/>
-    <hyperlink ref="B28" r:id="rId27" xr:uid="{4C1BA9E0-5C24-482B-895A-93E4FF6D7F94}"/>
-    <hyperlink ref="B29" r:id="rId28" xr:uid="{7F43F908-E262-4C52-A283-BC53176A8C46}"/>
-    <hyperlink ref="B31" r:id="rId29" xr:uid="{A55B142A-1F76-4FA4-8825-61B2F7CC0A1C}"/>
-    <hyperlink ref="B32" r:id="rId30" xr:uid="{C40CC3C2-AEB5-4CD8-88D8-C902A5085FAF}"/>
-    <hyperlink ref="B30" r:id="rId31" xr:uid="{3B59B242-3FBC-42FA-A878-6E97732489BB}"/>
+    <hyperlink ref="B22" r:id="rId21" xr:uid="{A430A9C6-FD58-4DE8-82B1-C2BDC43CD75D}"/>
+    <hyperlink ref="B23" r:id="rId22" xr:uid="{4BA87FC2-2482-47F3-AF0B-26573751D1D0}"/>
+    <hyperlink ref="B24" r:id="rId23" xr:uid="{CF736F36-5C13-46BF-8EFE-00A8F71CDBFA}"/>
+    <hyperlink ref="B25" r:id="rId24" xr:uid="{F3EE1F0F-3E4B-4FFA-A948-D718624032D3}"/>
+    <hyperlink ref="B26" r:id="rId25" xr:uid="{24CA94E5-1C41-4A90-8A88-F60639278F60}"/>
+    <hyperlink ref="B27" r:id="rId26" xr:uid="{4C1BA9E0-5C24-482B-895A-93E4FF6D7F94}"/>
+    <hyperlink ref="B28" r:id="rId27" xr:uid="{7F43F908-E262-4C52-A283-BC53176A8C46}"/>
+    <hyperlink ref="B30" r:id="rId28" xr:uid="{A55B142A-1F76-4FA4-8825-61B2F7CC0A1C}"/>
+    <hyperlink ref="B31" r:id="rId29" xr:uid="{C40CC3C2-AEB5-4CD8-88D8-C902A5085FAF}"/>
+    <hyperlink ref="B29" r:id="rId30" xr:uid="{3B59B242-3FBC-42FA-A878-6E97732489BB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
serialization and stocks for 2.8
</commit_message>
<xml_diff>
--- a/modules.xlsx
+++ b/modules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\josh\kenyaEMR-modules-updater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E490BAB4-124D-4B95-ADE7-261E9123F9DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1418CF-F7A3-45B7-954F-750C2A41E676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7576F9BB-DBC4-4D03-8B1C-D88545B56239}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="76">
   <si>
     <t>modules</t>
   </si>
@@ -254,6 +254,18 @@
   </si>
   <si>
     <t>version-2.55.0-snapshot</t>
+  </si>
+  <si>
+    <t>serialization</t>
+  </si>
+  <si>
+    <t>https://github.com/palladiumkenya/openmrs-module-serialization.xstream.git</t>
+  </si>
+  <si>
+    <t>stocks</t>
+  </si>
+  <si>
+    <t>stock-2.8.1-platform</t>
   </si>
 </sst>
 </file>
@@ -616,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D447332-634A-4264-831A-AFF551D7ED1B}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" bestFit="1" customWidth="1"/>
@@ -966,6 +978,28 @@
       </c>
       <c r="C31" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C33" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1001,6 +1035,8 @@
     <hyperlink ref="B30" r:id="rId28" xr:uid="{C40CC3C2-AEB5-4CD8-88D8-C902A5085FAF}"/>
     <hyperlink ref="B28" r:id="rId29" xr:uid="{3B59B242-3FBC-42FA-A878-6E97732489BB}"/>
     <hyperlink ref="B31" r:id="rId30" xr:uid="{9911E7B8-06C5-456A-9C67-209E377DE4D4}"/>
+    <hyperlink ref="B32" r:id="rId31" xr:uid="{8D06A38D-AAD3-41FE-BDFB-143E0E3CB246}"/>
+    <hyperlink ref="B33" r:id="rId32" xr:uid="{6A8AB9E9-C98F-411D-AEE3-133806E23CE8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>